<commit_message>
Nuevas entradas de bitácora, y tribu Bramasole.md
</commit_message>
<xml_diff>
--- a/recursos/ListadoGuardianes.xlsx
+++ b/recursos/ListadoGuardianes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Aetheon\recursos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{B51595AE-0806-4270-8AEB-260215F05E7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50CC526-FAC5-493C-9782-270CBA980373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BAE1CEE7-E3BE-48C7-8A25-E62C669B7CA3}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="131">
   <si>
     <t>Nombre</t>
   </si>
@@ -409,6 +409,30 @@
   </si>
   <si>
     <t>Olivo vecino del paseo del Rikudo Sennin, que no sólo es Guardián, sino en gran parte, ideólogo de la arquitectura del Codex de Aetheon</t>
+  </si>
+  <si>
+    <t>Evan</t>
+  </si>
+  <si>
+    <t>Almendro</t>
+  </si>
+  <si>
+    <t>Compañero de veladas, confesor inquebrantable, el que pacientemente espera en su cocina, con el café frío y sus pies descalzos.</t>
+  </si>
+  <si>
+    <t>El primero de una hilera de 5 almendros, que actualmente se haya talado, pero nuestra pretensión es plantar un nuevo almendro para completar esta ausencia.</t>
+  </si>
+  <si>
+    <t>Lorca</t>
+  </si>
+  <si>
+    <t>Keating</t>
+  </si>
+  <si>
+    <t>Whitman</t>
+  </si>
+  <si>
+    <t>Machado</t>
   </si>
 </sst>
 </file>
@@ -497,7 +521,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -508,9 +532,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -845,7 +867,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BFC84A5-5464-4015-A7CF-CFA3A9B03A73}">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -1407,10 +1429,10 @@
       <c r="B40" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="D40" s="11" t="s">
+      <c r="D40" s="8" t="s">
         <v>120</v>
       </c>
     </row>
@@ -1421,10 +1443,10 @@
       <c r="B41" t="s">
         <v>114</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" t="s">
         <v>116</v>
       </c>
-      <c r="D41" s="12" t="s">
+      <c r="D41" t="s">
         <v>121</v>
       </c>
     </row>
@@ -1435,11 +1457,57 @@
       <c r="B42" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="8" t="s">
         <v>122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A43" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B43" t="s">
+        <v>124</v>
+      </c>
+      <c r="C43" t="s">
+        <v>125</v>
+      </c>
+      <c r="D43" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B44" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B45" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A46" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A47" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="B47" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lo imposible en el espacio
</commit_message>
<xml_diff>
--- a/recursos/ListadoGuardianes.xlsx
+++ b/recursos/ListadoGuardianes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Git\Aetheon\recursos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E50CC526-FAC5-493C-9782-270CBA980373}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE7E8DA3-8AE1-4497-BE47-3A9F4027B576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BAE1CEE7-E3BE-48C7-8A25-E62C669B7CA3}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="139">
   <si>
     <t>Nombre</t>
   </si>
@@ -426,20 +426,64 @@
     <t>Lorca</t>
   </si>
   <si>
-    <t>Keating</t>
-  </si>
-  <si>
-    <t>Whitman</t>
-  </si>
-  <si>
     <t>Machado</t>
+  </si>
+  <si>
+    <t>No son todos realmente poetas, alguno de elllos ni siquiera murió, pero la referencia, creo que es obvia</t>
+  </si>
+  <si>
+    <t>Nunca se atrevieron a imaginar que el cosmos / Está vivo en sí mismo, y tiene un significado tan cercano, Entonces lo que regrese intacto serán aquellos que / Supieron cómo aferrarse a lo bueno y lo verdadero</t>
+  </si>
+  <si>
+    <t>Carpe Diem, Las palabras y las ideas pueden cambiar el mundo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Me celebro y me canto a mí mismo, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Oh Capitán! Mi Capitán!</t>
+    </r>
+  </si>
+  <si>
+    <t>Caminante no hay camino, Anoche cuando dormía, donde sueña que una fontana o un ardiente sol fluyen dentro de su corazón, Todo pasa y todo queda; / pero lo nuestro es pasar, / pasar haciendo caminos, / caminos sobre la mar</t>
+  </si>
+  <si>
+    <t>Verde que te quiero verde, La muerte / entra y sale / de la taberna, El lagarto está llorando. / El lagarto y la lagartarga / tienen su delantalito blanco</t>
+  </si>
+  <si>
+    <t>Mistral</t>
+  </si>
+  <si>
+    <t>Neruda</t>
+  </si>
+  <si>
+    <t>Walt</t>
+  </si>
+  <si>
+    <t>Otro Poeta muerto, Esta lista de nombres, enumera referentes. Evan Mantyk, Federico Garcia Lorca, Pablo Neruda, Walt Whitman, Antonio Machado, Gabriela Mistral</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,6 +495,14 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -521,7 +573,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -533,6 +585,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -867,12 +921,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BFC84A5-5464-4015-A7CF-CFA3A9B03A73}">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="91.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.5703125" customWidth="1"/>
     <col min="4" max="4" width="85.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1324,7 +1378,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>90</v>
       </c>
@@ -1338,7 +1392,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>93</v>
       </c>
@@ -1352,7 +1406,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>96</v>
       </c>
@@ -1366,7 +1420,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>99</v>
       </c>
@@ -1380,7 +1434,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>102</v>
       </c>
@@ -1394,7 +1448,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>106</v>
       </c>
@@ -1408,7 +1462,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>109</v>
       </c>
@@ -1422,7 +1476,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>113</v>
       </c>
@@ -1436,7 +1490,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
         <v>115</v>
       </c>
@@ -1450,7 +1504,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>118</v>
       </c>
@@ -1464,7 +1518,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
         <v>123</v>
       </c>
@@ -1477,37 +1531,90 @@
       <c r="D43" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E43" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>127</v>
       </c>
       <c r="B44" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C44" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B45" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C45" t="s">
+        <v>138</v>
+      </c>
+      <c r="D45" t="s">
+        <v>129</v>
+      </c>
+      <c r="E45" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B46" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="C46" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E46" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="10" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B47" t="s">
         <v>124</v>
+      </c>
+      <c r="C47" t="s">
+        <v>138</v>
+      </c>
+      <c r="D47" t="s">
+        <v>129</v>
+      </c>
+      <c r="E47" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>